<commit_message>
filter pull-quote comments that copy op verbatim
</commit_message>
<xml_diff>
--- a/Topic Relevant Comments - Nigeria/Agba John Doe/Never Leave Marriage Because Husband Cheated.xlsx
+++ b/Topic Relevant Comments - Nigeria/Agba John Doe/Never Leave Marriage Because Husband Cheated.xlsx
@@ -55,9 +55,6 @@
     <t>Man or woman, even the Bible permits divorce if cheating is involved. If you really love someone you can't be comfortable sharing them with someone else. One benefit of monogamy is to avoid catching stds, if hubby's distin is still for the community, what's the point? God abeg.</t>
   </si>
   <si>
-    <t>"A faithful husband is a disciplined husband but doesn't necessarily mean he's actually a good husband and father".</t>
-  </si>
-  <si>
     <t>What would be reduce from the life span of a man, if he decides to be a faithful husband? Can't they see their wife's are hurting and yet they derive pleasure in increasing the hurt with the excuse of "men are polygamous in nature" ‍♀️</t>
   </si>
   <si>
@@ -97,12 +94,12 @@
     <t>Chai! This marriage thing isn't for the faint hearted</t>
   </si>
   <si>
+    <t>Yes sir since being faithful is a farce let us stay with cheating men in peace,till they give us HIV or marry the side chick and be spiting us on social media with it,you too get sense walai</t>
+  </si>
+  <si>
     <t>Please..a woman who intend to get married and stay committed to it should read this tweet with all sense of sincerity &amp; open mind. Especially where sir Jon said THE CONSEQUENCES ARE NOT THE SAME FOR BOTH GENDER.</t>
   </si>
   <si>
-    <t>Yes sir since being faithful is a farce let us stay with cheating men in peace,till they give us HIV or marry the side chick and be spiting us on social media with it,you too get sense walai</t>
-  </si>
-  <si>
     <t>Sir John, I would like you to one day make a thread on domestic abuse from the man. Would really love to see your thoughts on that.</t>
   </si>
   <si>
@@ -139,12 +136,12 @@
     <t>The cheating or infidelity or I'll rather say polygamy is in the DNA of men originally designed and created by God are you ready to recreate another man ? Are you GOD?</t>
   </si>
   <si>
+    <t>I see a lot of men happily replying and seconding this tweet, now the tweet itself is a sad reality meaning that it holds true for majority. If you truly love your woman , you stay faithful, it breaks a woman and a lot of you can't even take it if your woman cheats on you,</t>
+  </si>
+  <si>
     <t>In as much as we Husbands wey get sense pray our marriages don't get this point, cheating is not the same for man and woman... Ask your mother, she will tell you to stand your ground, there is nothing for you outside there, na you go loose if you say you wan move...</t>
   </si>
   <si>
-    <t>I see a lot of men happily replying and seconding this tweet, now the tweet itself is a sad reality meaning that it holds true for majority. If you truly love your woman , you stay faithful, it breaks a woman and a lot of you can't even take it if your woman cheats on you,</t>
-  </si>
-  <si>
     <t>never fight your husband over another woman out there, she's very irrelevant, continue to be his peace and hiding place, he will get tired and come back home. A genuine born again Christian have much more deeper understanding of why he shouldn't cheat as a man, even the wife</t>
   </si>
   <si>
@@ -166,15 +163,15 @@
     <t>Ye lots that projects marriage as if men are doing women favor by being married to them. Motivational speaker wanna be.</t>
   </si>
   <si>
+    <t>Let me give u an original answer.Originally god never created man 2 b one man &amp;one woman.monogamy is a Western construct.A woman cant stand the libido of an average man. So from the biblical evidence will have more telling of that men in the Bible married so many women</t>
+  </si>
+  <si>
     <t>I know you're trying to tell us the sad reality of life, but the truth is some of us women are not strong enough to stomach the thought of infidelity. It will break us. Hopefully, God will give those of us who are still single, the ability to discern and choose principled men.</t>
   </si>
   <si>
     <t>Most Women leaving cheating partners end up as side chic/2nd wife,ironical isn't it? That's d reality on cheating,consequences is never same,A cheating woman will loose her marriage while a in most cases man will not as long as he protect,provide,secure and manage his home</t>
   </si>
   <si>
-    <t>Let me give u an original answer.Originally god never created man 2 b one man &amp;one woman.monogamy is a Western construct.A woman cant stand the libido of an average man. So from the biblical evidence will have more telling of that men in the Bible married so many women</t>
-  </si>
-  <si>
     <t>At first when I began to read, it makes sense. Mr. John with all due respect, it will be respectful to women to encourage them to stay committed to their marriage for more Godly reasons, e.g; none of our Godly mother like Sarah left Abraham for cheating. Infact, I say this a lot,</t>
   </si>
   <si>
@@ -184,12 +181,12 @@
     <t>At the end those side chics would still leave you,and that's for a fact.I've always said this and I'll keep saying it " an average male child is not properly trained" why would you be married and all you can think of is how to betray your familyGod pls help me be a good husband</t>
   </si>
   <si>
+    <t>Thanks bro, u nailed it✅ I pray God should give me more patient in marriage when i marry</t>
+  </si>
+  <si>
     <t>Be calm pretty posh, Nobody is glorifying CHEATING HERE... Have you ever asked yourself why MEN can marry as many women as them like but a WOMAN can't marry many MEN as she can If you can answer the question, then FINE</t>
   </si>
   <si>
-    <t>Thanks bro, u nailed it✅ I pray God should give me more patient in marriage when i marry</t>
-  </si>
-  <si>
     <t>"so on judgement day" the two religions that preaches this also preaches that one man can marry more than one wife. So what judgement is there to be passed again?</t>
   </si>
   <si>
@@ -265,63 +262,60 @@
     <t>I don't support cheating by any means but a psychologist on TEDX once said that; Men cheat to KEEP their marriage, WOMEN cheat to leave their marriage. A man just need a place to cheat, but women need a reason to cheat. That's why a cheating woman should never be let back in.</t>
   </si>
   <si>
+    <t>Sadly true, but I can't help think that this only just adds to giving some men the license and validity to cheat, rub it in the face of the wife and expect her to persevere because she can be easily replaced.</t>
+  </si>
+  <si>
     <t>And sincerely this is one of the beauty of salvation.. No believing man will cheat on you.. It's not about morals for such a man rather it's about eternal life and self worth. Joseph(s) don't fall for beauties no matter the shapes. They consider it a sin against God..</t>
   </si>
   <si>
-    <t>Sadly true, but I can't help think that this only just adds to giving some men the license and validity to cheat, rub it in the face of the wife and expect her to persevere because she can be easily replaced.</t>
-  </si>
-  <si>
     <t>That's bitter truth , but men can do better and work on their self discipline. Because the women have started to cheat back which leads to " men bringing up children that are not theirs " DNA palaver up and down</t>
   </si>
   <si>
+    <t>I just feel in as much as your marriage is peaceful, accomodating, everything is going on smoothly and u r happy as a lady in it, don't seek for a second. I know how painful and frustrating it can be if you see your partner cheating, but if he doesn't do it in from of u, or he</t>
+  </si>
+  <si>
+    <t>this comment! like they think all women can endure cheating..my dad was a serial cheat and i know how my mum was feeling before she died..and i can never ever endure like my mum..never!i will rather be alone than endure nonsense..my happiness and my sanity comes first.</t>
+  </si>
+  <si>
+    <t>So in other words, cheating is healthy and men should do it more?? Or they should still try and be decent with their ways??</t>
+  </si>
+  <si>
     <t>So what about situation were the cheating partner get his /her partner infected of a STD???</t>
   </si>
   <si>
-    <t>I just feel in as much as your marriage is peaceful, accomodating, everything is going on smoothly and u r happy as a lady in it, don't seek for a second. I know how painful and frustrating it can be if you see your partner cheating, but if he doesn't do it in from of u, or he</t>
-  </si>
-  <si>
-    <t>So in other words, cheating is healthy and men should do it more?? Or they should still try and be decent with their ways??</t>
-  </si>
-  <si>
-    <t>this comment! like they think all women can endure cheating..my dad was a serial cheat and i know how my mum was feeling before she died..and i can never ever endure like my mum..never!i will rather be alone than endure nonsense..my happiness and my sanity comes first.</t>
-  </si>
-  <si>
-    <t>I want to put it on my whatssap status but Feminist will come for me and I'm tired for an argument. This is wisdom</t>
-  </si>
-  <si>
     <t>Every next generation makes the mistake of assuming they are smarter than the previous ones. There are curtains that would have protected women socially that women have ripped off now. It's gender equality, may the best human win.</t>
   </si>
   <si>
     <t>Majorly men cheat because they don't get what they want from their women and they can't change them to what they want. In some cases you will find out that the man married the body he desire but not the soul he wanted. Then he would go in search of the one that suit his fantasy</t>
   </si>
   <si>
+    <t>Women and men will never be the same.. This will forever exist without going into extinction. Just like saying racism will stop, we all know surely it will exist directly or indirectly. Men will always cheat no matter what! 98% of rich married men cheats..</t>
+  </si>
+  <si>
     <t>Are you encouraging men to keep cheating ?</t>
   </si>
   <si>
-    <t>Women and men will never be the same.. This will forever exist without going into extinction. Just like saying racism will stop, we all know surely it will exist directly or indirectly. Men will always cheat no matter what! 98% of rich married men cheats..</t>
-  </si>
-  <si>
     <t>Just by reading comments, men feel happy that u ve made this thread. Women who wish to remain committed to their cheating partner must learn to substitute love for money/wealth. If ur hubby doesn't cater for u/children and u do not earn more by being married, please leave!</t>
   </si>
   <si>
+    <t>Know this and know peace. Not all men cheat. Not all African men cheat. Any man can cheat African or asian. Don't marry a man that cheats and give excuse that all men cheat! You have bought the Lie of the devil.He is the father of all Liars! Run from cheats from d onset</t>
+  </si>
+  <si>
     <t>Clearly it is evident in our societal response. Omo it require deep thoughts before a woman must leave her marriage otherwise she'll end up regretting her actions for the rest of her entire life if she can't find what she once had, and the reality that she can never find it. Hmm</t>
   </si>
   <si>
-    <t>Know this and know peace. Not all men cheat. Not all African men cheat. Any man can cheat African or asian. Don't marry a man that cheats and give excuse that all men cheat! You have bought the Lie of the devil.He is the father of all Liars! Run from cheats from d onset</t>
-  </si>
-  <si>
     <t>Who do men cheat with? Is it not women.</t>
   </si>
   <si>
+    <t>While I find everything written here understandable, I still think a cheating husband deserves some kind of punishment from his wife. At least something to make him not want to do it another time. Repeating this act is however evil and shouldn't be seen as normal no matter what.</t>
+  </si>
+  <si>
     <t>It depends bro. It the man cheats and still beats up the wife, that wife deserves to leave. It all depend on the kind of marriage you find yourself into. What is stopping most marriages from collapsing is the children</t>
   </si>
   <si>
     <t>Being committed means being safe n happy in a relationship bt enduring, especially in this century of men,is something I will not subscribed for anybody including my sis even if the man in question is my brother,I will not take it from him cause that is how most ⏬</t>
   </si>
   <si>
-    <t>While I find everything written here understandable, I still think a cheating husband deserves some kind of punishment from his wife. At least something to make him not want to do it another time. Repeating this act is however evil and shouldn't be seen as normal no matter what.</t>
-  </si>
-  <si>
     <t>The only time I can suggest divorce is when the marriage is abusive aside that no go divorce over cheating ooo especially for the ladies. It doesn't end well</t>
   </si>
   <si>
@@ -385,12 +379,12 @@
     <t>Most times when people call off relationships, it's not just the cheating, there's more</t>
   </si>
   <si>
+    <t>Testosterone na your mate? Imagine your wife is on birth control pills which reduces the release of their sex hormones but your Testosterone is running on auto pilot. Every morning you wake up with hard dick. You're a ticking time bomb to the fidelity world. That's where</t>
+  </si>
+  <si>
     <t>Lesson: don't leave your man/husband because of rain, it rains everywhere. This is just reality of life. I can't fight or leave because of another woman, I believe he is an adult and he knows what is good for him.</t>
   </si>
   <si>
-    <t>Testosterone na your mate? Imagine your wife is on birth control pills which reduces the release of their sex hormones but your Testosterone is running on auto pilot. Every morning you wake up with hard dick. You're a ticking time bomb to the fidelity world. That's where</t>
-  </si>
-  <si>
     <t>I know of a wife who was too feminist. The guy went on to put a ring on his side chick and the first wife with a traditional marriage is now the side chick. He visits her here n there</t>
   </si>
   <si>
@@ -430,18 +424,18 @@
     <t>I had woke thoughts until I realised that I just didn't want to accept the painful things @jon_d_doe said. That some realities are painful makes them no less realities. I would choose to be celibate if I find myself with a cheating husband. They're not worth being sad in a union.</t>
   </si>
   <si>
+    <t>Not only married women. Dating women too. The more "exes" you're accumulating. The lesser the men that finds interest in you.</t>
+  </si>
+  <si>
+    <t>Yes sir, u just reveal the whole truth about inter sexual relationship. Women can never be like men. Men are polygamous in nature, and don't forget men are always horny due to high testosterone.</t>
+  </si>
+  <si>
+    <t>It's very funny how people think. So what if this said husband is late sef, won't the woman survive??? Why do men feel women should be cheated on as a right? How will you father's feel if your little girl gets married and the husband turns out to push her to depression???</t>
+  </si>
+  <si>
     <t>Last 2 years my neighbor's wife left because she noticed that he cheated. Not long after that lockdown start baba start making out with another lady in the next compound words got to the wife where she was staying with her family at ikorodu babe return baba say he no marry again</t>
   </si>
   <si>
-    <t>Not only married women. Dating women too. The more "exes" you're accumulating. The lesser the men that finds interest in you.</t>
-  </si>
-  <si>
-    <t>Yes sir, u just reveal the whole truth about inter sexual relationship. Women can never be like men. Men are polygamous in nature, and don't forget men are always horny due to high testosterone.</t>
-  </si>
-  <si>
-    <t>It's very funny how people think. So what if this said husband is late sef, won't the woman survive??? Why do men feel women should be cheated on as a right? How will you father's feel if your little girl gets married and the husband turns out to push her to depression???</t>
-  </si>
-  <si>
     <t>I always ask, if all men cheat or all men are dogs why will u leave your man for another man?</t>
   </si>
   <si>
@@ -460,12 +454,12 @@
     <t>I do tell ladies dat, man can cheat on u &amp; still love u with every breath. They do not understand how it works,Man sees love diff from sex they are not synonymous but women thinks a man that love her shouldnt cheat on ha.Man can be committed.</t>
   </si>
   <si>
+    <t>Lol. I'm just happy that women are slowly beginning to be independent and choosy. Because this was legit the scum they fed our mothers. Thats why sugar daddy is now a culture. Grown, married, men disgustingly preying on young girls while leaving their wives miserable</t>
+  </si>
+  <si>
     <t>When he had a thread about women being committed to their emotions and not men's sacrifices, the women were clapping for him. Now that he has also talked about reality of the consequences of cheating not being the same for a man and a woman una wan chop am raw!! .. Choo!! ‍♂️</t>
   </si>
   <si>
-    <t>Lol. I'm just happy that women are slowly beginning to be independent and choosy. Because this was legit the scum they fed our mothers. Thats why sugar daddy is now a culture. Grown, married, men disgustingly preying on young girls while leaving their wives miserable</t>
-  </si>
-  <si>
     <t>I ask again....if she decides to leave will she remain celibate? If not who will she pick? A younger man who will be faithful to her? Another man who will carry all her responsibilities and be faithful to her?.... If your answer is same as he has typed, then he's not wrong.</t>
   </si>
   <si>
@@ -475,15 +469,15 @@
     <t>Most divorced women of African descent end up bring past around like footballs while the man ends up in a stable relationship/marriage. Don't leave your husband for the streets sistas‍♂️‍♂️‍♂️</t>
   </si>
   <si>
+    <t>Truth, we had this argument on a women group once, myself and some women are of this opinion, not everything divorce your husband and after divorce you will become the reason you left your home in another woman's marriage. A divorce woman can rarely marry a fresh man but some...</t>
+  </si>
+  <si>
     <t>We've heard you sir There's no problem just keep this same energy when your sister gets cheated on and probably gets and STI from her husband</t>
   </si>
   <si>
     <t>Value sir .....thank u for this community I have be able to learn a lot Men and women does not have the same grace when dey cheat</t>
   </si>
   <si>
-    <t>Truth, we had this argument on a women group once, myself and some women are of this opinion, not everything divorce your husband and after divorce you will become the reason you left your home in another woman's marriage. A divorce woman can rarely marry a fresh man but some...</t>
-  </si>
-  <si>
     <t>This is the sad reality. There was this man in our business line he was cheating on the wife then one of his boys told the wife and the wife confronted the husband shouting, threatening and all that, the moment the man found out who told her he first of all sent the boy away</t>
   </si>
   <si>
@@ -499,12 +493,12 @@
     <t>How is a woman supposed to stop a man from cheating? Is she supposed to flog him? How? So as an adult man that you are, you realize that cheating is not good but you continue and then you're expecting the woman to be to the one stop you. Why can't you stop yourself? Na wah o.</t>
   </si>
   <si>
+    <t>Husband get protected, If you choose to stay please get tested frequently too. Recently came across a petition where the husband infected the wife wit HIV, her family had to speak to her to stay since they were both infected and sent the kids off abroad so dy don't get infected.</t>
+  </si>
+  <si>
     <t>A thread like this resonates with life and reality, you can't find this undiluted truth anywhere, if you like heed to it, if you like don't, it's either you learn to live or live to perish.</t>
   </si>
   <si>
-    <t>Husband get protected, If you choose to stay please get tested frequently too. Recently came across a petition where the husband infected the wife wit HIV, her family had to speak to her to stay since they were both infected and sent the kids off abroad so dy don't get infected.</t>
-  </si>
-  <si>
     <t>He's not encouraging men to cheat. It's a sad reality</t>
   </si>
   <si>
@@ -520,12 +514,12 @@
     <t>Find out if he's cheating with 9in10.com, then leave Sis</t>
   </si>
   <si>
+    <t>I read the write up till the end, not all your points are valid man, you're making it sound like African women are very primitive... But your view towards women make me feel like you think they lack self esteem... Everyone has his or her marital story don't make it sound like a</t>
+  </si>
+  <si>
     <t>@mrjohndoe... Are you now saying, even in a abusive marriage, make she stay, abusive marriage dat de husband s beating her nd cheating on her,... Wah will u say abut dat</t>
   </si>
   <si>
-    <t>I read the write up till the end, not all your points are valid man, you're making it sound like African women are very primitive... But your view towards women make me feel like you think they lack self esteem... Everyone has his or her marital story don't make it sound like a</t>
-  </si>
-  <si>
     <t>Why leave a cheating spouse when you can stay and ruin his life</t>
   </si>
   <si>
@@ -535,12 +529,12 @@
     <t>Lmao better to be a sleeping around woman than be with a "Husband" who goes around disrespecting WIFEE sleeping with anything sleepable. Make everywhere scatter!</t>
   </si>
   <si>
+    <t>Hard truth, watch how they will twist this into; he's encouraging cheating.</t>
+  </si>
+  <si>
     <t>A lot of facts here are better imagined than experienced. When you sit down with older ladies who left their husbands for little issues that could be managed, now they're begging for just a night together with a man who doesn't have their time. There's money no companionship.Sad!</t>
   </si>
   <si>
-    <t>Hard truth, watch how they will twist this into; he's encouraging cheating.</t>
-  </si>
-  <si>
     <t>Will men please stop cheating for crying out loud!!! Nawa ooo</t>
   </si>
   <si>
@@ -604,12 +598,12 @@
     <t>I had a client who filed for divorce bcos a man she was dating asked her to so that they could be free to marry. I finished the case &amp; got the marriage dissolved. Years later, I met d lady that referred her to me &amp; asked her if the man eventually married my client.She said no.</t>
   </si>
   <si>
+    <t>Is it all about servicing and getting serviced just to survive? If she get money nko? Una go just dey think one way. If she wan dey with another man wey get woman nko? What if that's what she want?</t>
+  </si>
+  <si>
     <t>But. The white ladies leave their cheating husband and claim his properties, they have a social system that forces the man to still provide for the kids. We no get am here, yet we wan copy them, say na wokeness.</t>
   </si>
   <si>
-    <t>Is it all about servicing and getting serviced just to survive? If she get money nko? Una go just dey think one way. If she wan dey with another man wey get woman nko? What if that's what she want?</t>
-  </si>
-  <si>
     <t>Ladies should not be afraid of change. You don't know how to be alone so you'd rather stay and get infected. If you can't stand it leave Africa there are countries in need of women even though I might not leave my husband due to him cheating.</t>
   </si>
   <si>
@@ -617,6 +611,12 @@
   </si>
   <si>
     <t>You can say it in public that your father is a cheater and sleeps around, you can't say that for your mother. That's all. Thanks for reading</t>
+  </si>
+  <si>
+    <t>We all feel hurt when mistreated. So to the men singing praises to this, I hope you maintain the same energy if she cheats back, you totally asked for it, Idk about anyone else but I'd rather leave a cheating man than cheat back on him, I'd be doing a great dishonor to myself,</t>
+  </si>
+  <si>
+    <t>Comrade, please break this thing down for me. You mean side chick turn wife and wife turn side chick Abi na eye dey pain me?</t>
   </si>
 </sst>
 </file>

</xml_diff>